<commit_message>
feat: add formula validation and preview Co-authored-by: monkeycode-ai <monkeycode-ai@chaitin.com>
</commit_message>
<xml_diff>
--- a/sample_data/complex_template_200x15.xlsx
+++ b/sample_data/complex_template_200x15.xlsx
@@ -9,10 +9,12 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="销售明细" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="区域字典" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'销售明细'!$A$1:$O$201</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'汇总'!$A$1:$C$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'汇总'!$A$1:$E$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'区域字典'!$A$1:$C$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -4748,12 +4750,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4772,6 +4776,16 @@
           <t>order_count</t>
         </is>
       </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>region_level</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>owner_hint</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -4784,7 +4798,15 @@
         <v/>
       </c>
       <c r="C2">
-        <f>COUNTIF(销售明细!D$2:D$201,A2)</f>
+        <f>COUNTIFS(销售明细!D$2:D$201,A2,销售明细!N$2:N$201,"正常")</f>
+        <v/>
+      </c>
+      <c r="D2">
+        <f>IFERROR(VLOOKUP(A2,区域字典!$A:$B,2,FALSE),"未知")</f>
+        <v/>
+      </c>
+      <c r="E2">
+        <f>IFERROR(XLOOKUP(A2,区域字典!$A:$A,区域字典!$C:$C),"未配置")</f>
         <v/>
       </c>
     </row>
@@ -4799,7 +4821,15 @@
         <v/>
       </c>
       <c r="C3">
-        <f>COUNTIF(销售明细!D$2:D$201,A3)</f>
+        <f>COUNTIFS(销售明细!D$2:D$201,A3,销售明细!N$2:N$201,"正常")</f>
+        <v/>
+      </c>
+      <c r="D3">
+        <f>IFERROR(VLOOKUP(A3,区域字典!$A:$B,2,FALSE),"未知")</f>
+        <v/>
+      </c>
+      <c r="E3">
+        <f>IFERROR(XLOOKUP(A3,区域字典!$A:$A,区域字典!$C:$C),"未配置")</f>
         <v/>
       </c>
     </row>
@@ -4814,7 +4844,15 @@
         <v/>
       </c>
       <c r="C4">
-        <f>COUNTIF(销售明细!D$2:D$201,A4)</f>
+        <f>COUNTIFS(销售明细!D$2:D$201,A4,销售明细!N$2:N$201,"正常")</f>
+        <v/>
+      </c>
+      <c r="D4">
+        <f>IFERROR(VLOOKUP(A4,区域字典!$A:$B,2,FALSE),"未知")</f>
+        <v/>
+      </c>
+      <c r="E4">
+        <f>IFERROR(XLOOKUP(A4,区域字典!$A:$A,区域字典!$C:$C),"未配置")</f>
         <v/>
       </c>
     </row>
@@ -4829,7 +4867,15 @@
         <v/>
       </c>
       <c r="C5">
-        <f>COUNTIF(销售明细!D$2:D$201,A5)</f>
+        <f>COUNTIFS(销售明细!D$2:D$201,A5,销售明细!N$2:N$201,"正常")</f>
+        <v/>
+      </c>
+      <c r="D5">
+        <f>IFERROR(VLOOKUP(A5,区域字典!$A:$B,2,FALSE),"未知")</f>
+        <v/>
+      </c>
+      <c r="E5">
+        <f>IFERROR(XLOOKUP(A5,区域字典!$A:$A,区域字典!$C:$C),"未配置")</f>
         <v/>
       </c>
     </row>
@@ -4844,8 +4890,138 @@
         <v/>
       </c>
       <c r="C6">
-        <f>COUNTIF(销售明细!D$2:D$201,A6)</f>
-        <v/>
+        <f>COUNTIFS(销售明细!D$2:D$201,A6,销售明细!N$2:N$201,"正常")</f>
+        <v/>
+      </c>
+      <c r="D6">
+        <f>IFERROR(VLOOKUP(A6,区域字典!$A:$B,2,FALSE),"未知")</f>
+        <v/>
+      </c>
+      <c r="E6">
+        <f>IFERROR(XLOOKUP(A6,区域字典!$A:$A,区域字典!$C:$C),"未配置")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E6"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>region</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>region_level</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>华东</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>核心区域</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>区域负责人-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>华南</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>成长区域</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>区域负责人-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>华北</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>核心区域</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>区域负责人-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>西南</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>成长区域</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>区域负责人-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>西北</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>核心区域</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>区域负责人-05</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>